<commit_message>
Add explicit policy citation links
</commit_message>
<xml_diff>
--- a/02_元数据/知识库管理工作簿.xlsx
+++ b/02_元数据/知识库管理工作簿.xlsx
@@ -12,25 +12,27 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工核验表" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="政策资料台账" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则清单" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地区覆盖清单" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待采集链接" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索评测结果" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全文检索结果" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标题清洗建议" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="政策关联关系" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地区覆盖清单" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待采集链接" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索评测结果" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全文检索结果" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标题清洗建议" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'问题评测表'!$A$1:$R$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'人工核验表'!$A$1:$Z$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'政策资料台账'!$A$1:$V$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'规则清单'!$A$1:$R$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'来源清单'!$A$1:$P$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'地区覆盖清单'!$A$1:$J$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'待采集链接'!$A$1:$L$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'检索评测结果'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'全文检索结果'!$A$1:$Q$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'标题清洗建议'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'政策关联关系'!$A$1:$M$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'来源清单'!$A$1:$P$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'地区覆盖清单'!$A$1:$J$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'待采集链接'!$A$1:$L$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'检索评测结果'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'全文检索结果'!$A$1:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'标题清洗建议'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -484,7 +486,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 18:39</t>
+          <t>2026-04-27 10:16</t>
         </is>
       </c>
     </row>
@@ -575,41 +577,53 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>来源清单</t>
+          <t>政策关联关系</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>用于控制自动采集的白名单来源。</t>
+          <t>仅记录新政策明文引用旧政策的关系，用于搜索页库内跳转和版本脉络核验。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>地区覆盖清单</t>
+          <t>来源清单</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>用于查看省级、直辖市、副省级城市和电网经营区覆盖情况。</t>
+          <t>用于控制自动采集的白名单来源。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>地区覆盖清单</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>用于查看省级、直辖市、副省级城市和电网经营区覆盖情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>待采集链接</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>用于人工确认后交给采集脚本下载入库。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -620,209 +634,1096 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>检索时间</t>
+          <t>评测编号</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>查询词</t>
+          <t>问题</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>排序</t>
+          <t>标准依据文件</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>得分</t>
+          <t>Top1资料编号</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>资料编号</t>
+          <t>Top1标题</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>文件标题</t>
+          <t>Top1得分</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>发布部门</t>
+          <t>Top3标题</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>采集来源机构</t>
+          <t>Top3命中</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>发布日期</t>
+          <t>标准文件是否已入库</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>文号</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>适用地区</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>来源类型</t>
-        </is>
-      </c>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>市场主题</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="inlineStr">
-        <is>
-          <t>权威等级</t>
-        </is>
-      </c>
-      <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>有效状态</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
-        <is>
-          <t>原文链接</t>
-        </is>
-      </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>命中说明</t>
+          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 18:36</t>
+          <t>Q-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>国能发监管规</t>
+          <t>全国统一电力市场体系建设的主要目标是什么</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>关于加快建设全国统一电力市场体系的指导意见</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>13.00</t>
+          <t>AUTO-20260424-FD9AA2BEA1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>49.00</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家能源局关于印发《电力市场注册基本规则》的通知</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Q-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>电力市场注册基本规则对经营主体注册提出了哪些要求</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>电力市场注册基本规则</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>AUTO-20260424-2ABE953CDD</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>国家能源局关于印发《电力市场注册基本规则》的通知</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2024-09-13</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>国能发监管规〔2024〕76号</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>全国</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>官方政策</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>电力市场;中长期;现货;辅助服务</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>现行有效</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>https://zfxxgk.nea.gov.cn/2024-09/13/c_1212399683.htm</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>国能发监管规:文号</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>47.00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局关于印发《电力市场注册基本规则》的通知 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Q-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则中市场成员包括哪些类型</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>37.00</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Q-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>省间电力现货交易规则修订主要涉及哪些内容</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>关于修订省间电力现货交易规则的复函</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-55178B2DFC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>【关于修订省间电力现货交易规则的复函(发改办体改〔2026〕275号)】-国家发展和改革委员会</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>65.00</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>【关于修订省间电力现货交易规则的复函(发改办体改〔2026〕275号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Q-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>华中区域省间电力中长期市场实施细则适用于哪些交易范围</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>华中区域省间电力中长期市场实施细则</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-97CB3F74FC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>55.00</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知 | 关于公开征求《华中区域省间电力中长期交易实施细则（征求意见稿）》意见的通知 | 关于印发《重庆市电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>湖北省电力中长期市场实施细则规定了哪些主要交易类型</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>湖北省电力中长期市场实施细则</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-663B4D5B07</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《湖北省电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>49.00</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《湖北省电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>山东电力市场规则试行文件中中长期和现货如何衔接</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>山东电力市场规则(试行)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-2321F82FD1</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>关于山东电力现货市场由试运行转正式运行的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>31.50</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>关于山东电力现货市场由试运行转正式运行的通知_国家能源局山东监管办公室 | 《山东电力市场规则(试行)》编制说明_国家能源局山东监管办公室 | 关于印发《山东电力市场规则(试行)》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Q-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>山东并网运行和辅助服务管理实施细则涉及哪些主体和费用机制</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>山东省电力并网运行管理实施细则;山东省电力辅助服务管理实施细则</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-08F5111897</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>43.00</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室 | 关于印发《山东省电力并网运行管理实施细则》、《山东省电力辅助服务管理实施细则》的通知_国家能源局山东监管办公室 | 关于公开征求《山东省电力并网运行管理实施细则(征求意见稿)》《山东省电力辅助服务管理实施细则(征求意见稿)》意见的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Q-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>南方区域中长期电能量交易实施细则规定的交易组织方式有哪些</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>南方区域电力市场中长期电能量交易实施细则</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-E89DAD0775</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>南方区域电力市场中长期电能量交易实施细则等5项实施细则</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>40.50</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>南方区域电力市场中长期电能量交易实施细则等5项实施细则 | 关于加强辖区中长期批发交易合同签约履约监管的通知 | 电力市场信息披露基本规则（国能发监管〔2024〕9号）</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Q-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>辅助服务市场基本规则对辅助服务品种和结算提出了哪些要求</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>电力辅助服务市场基本规则</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-54244C417B</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>【关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)】-国家发展和改革委员会</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>37.00</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>【关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 关于印发《电力辅助服务市场基本规则》的通知</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q2"/>
+  <autoFilter ref="A1:J11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>检索时间</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>查询词</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>排序</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>得分</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>资料编号</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>文件标题</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>发布部门</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>采集来源机构</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>发布日期</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>文号</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>适用地区</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>来源类型</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>市场主题</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>权威等级</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>有效状态</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>原文链接</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>命中说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:40</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>南方区域 电力市场 运行规则</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-A4374A2C3D</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《南方区域电力市场运行规则（试行，2025年V1.0版）》的通知</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局派出机构</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局南方监管局</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>南方区域</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>监管规则</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>电力市场</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>试行</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>https://nfj.nea.gov.cn/xwzx/tzgg/202506/t20250625_283322.html</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>南方区域:标题/地区/备注;电力市场:标题/主题/关键词/备注;运行规则:标题/备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:40</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>南方区域 电力市场 运行规则</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>62.50</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-E89DAD0775</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>南方区域电力市场中长期电能量交易实施细则等5项实施细则</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>广州电力交易中心</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>广州电力交易中心</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-22</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>南方区域</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>交易规则</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>电力市场;中长期</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>现行有效</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gzpec.cn/law/jygz/202506/t20250624_34712.html</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>南方区域:标题/地区/备注;电力市场:标题/主题/关键词/备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:40</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>南方区域 电力市场 运行规则</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>59.50</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-02AD665464</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>关于印发南方区域电力市场配套实施细则的通知</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>广州电力交易中心</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>广州电力交易中心</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2024-11-14</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>南方区域</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>交易规则</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>现行有效</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gzpec.cn/law/jygz/202502/t20250214_34019.html</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>南方区域:标题/地区/备注;电力市场:标题/主题/关键词/备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:40</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>南方区域 电力市场 运行规则</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-BD09FE2823</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《南方区域新能源参与电力市场交易实施方案（试行）》的通知</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局派出机构</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局南方监管局</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>南方区域</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>监管规则</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>电力市场;新能源</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>试行</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>https://nfj.nea.gov.cn/xwzx/tzgg/202601/t20260104_293533.html</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>南方区域:标题/地区/备注;电力市场:标题/主题/关键词/备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:40</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>南方区域 电力市场 运行规则</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-991CDC4524</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《广东、广西、海南发电机组参与电力市场交易业务衔接暂行规定》的通知</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局派出机构</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局南方监管局</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>南方区域</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>监管规则</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>电力市场</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>现行有效</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>https://nfj.nea.gov.cn/xwzx/tzgg/202512/t20251224_292993.html</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>南方区域:地区;电力市场:标题/主题/关键词/备注</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19577,6 +20478,1900 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>关系编号</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>新政策资料编号</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>新政策标题</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>新政策发布日期</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>旧政策资料编号</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>旧政策标题</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>旧政策发布日期</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>关联类型</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>匹配依据</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>证据文本</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>置信度</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>是否人工确认</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>REL-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-D49D5FABE6</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《重庆市电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>电力用户，相关经营主体： 为贯彻落实加快建设全国统一电力市场要求，进一步深化重庆电力中长期市场建设，规范电力中长期交易行为，适应重庆电力市场高质量发展需要，依据《电力市场运行基本规则》（国家发展和改革委员会令 2024 年第 20 号）、《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>REL-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-A74926FCBF</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《江西省电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>电力用户，相关经营主体： 为贯彻落实加快建设全国统一电力市场要求，进一步深化江西电力中长期市场建设，规范电力中长期交易行为，适应江西电力市场高质量发展需要，依据《电力市场运行基本规则》（国家发展和改革委员会令 2024 年第 20 号）、《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>REL-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-712572408D</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《西藏自治区电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>电力用户，相关经营主体： 为贯彻落实加快建设全国统一电力市场要求，进一步深化西藏电力中长期市场建设，规范电力中长期交易行为，适应西藏电力市场高质量发展需要，依据《电力市场运行基本规则》（国家发展和改革委员会令 2024 年第 20 号）、《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>REL-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-663B4D5B07</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《湖北省电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>电力用户，相关经营主体： 为贯彻落实加快建设全国统一电力市场要求，进一步深化湖北电力中长期市场建设，规范电力中长期交易行为，适应湖北电力市场高质量发展需要，依据《电力市场运行基本规则》（国家发展和改革委员会令 2024 年第 20 号）、《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>REL-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-97CB3F74FC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-F67BBBF923</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>【关于印发《电力中长期市场基本规则》的通知(发改能源规〔2025〕1656号)】-国家发展和改革委员会</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力中长期市场基本规则</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>，相关经营主体 ： 为贯彻落实加快建设全国统一电力市场要求，进 一步深化华中区域省间电力中长期市场建设，规范省间电力中长期交易行为，依据《电力市场运行基本规则》《电力中长期市场基本规则》等有关规定，结合华中区域电力市场运行实际，华中能源监管局会同河南、湖南、四川能源监管办，组织电力交易机构修订形成《华中区域省间电力中长期市场实施细则》，经广泛征</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>REL-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-97CB3F74FC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>、电力交易机构、发电企业，相关经营主体 ： 为贯彻落实加快建设全国统一电力市场要求，进 一步深化华中区域省间电力中长期市场建设，规范省间电力中长期交易行为，依据《电力市场运行基本规则》《电力中长期市场基本规则》等有关规定，结合华中区域电力市场运行实际，华中能源监管局会同河南、湖南、四川能源监管办，组织电力交易机构修订形成《华中区域省间电力中长</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>REL-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-9A3E9D6FC0</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《山东电力市场监管办法(征求意见稿)》等意见的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>字体： 小 | 中 | 大 为贯彻落实国家有关部署，适应电力市场发展新形势，进一步规范山东电力市场秩序，完善监管机制，根据《电力监管条例》《电力市场监管办法》《电力市场运行基本规则》以及有关法律法规和政策规定，结合我省电力市场发展实际，我办组织有关单位对《山东电力市场监管办法(试行)》进行了修订，并同步编制了2项配套监管指引，现向社会公开征</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>REL-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-D8A4A0C9BE</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《华中区域省间电力中长期交易实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>局 Aa 字体： 小 | 中 | 大 为加快全国统一电力市场建设，进一步规范和完善华中区域电力中长期市场建设运营，维护区域电力市场秩序和经营主体合法权益， 根据《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会令第 20 号）《国家发展改革委 国家能源局关于印发&lt;电力中长期市场基本规则&gt;的通知》（发改能源规 〔2025〕1656 号</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>REL-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-63755B61E4</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《西藏自治区电力中长期市场实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>局华中监管局 Aa 字体： 小 | 中 | 大 为加快全国统一电力市场建设，进一步规范和完善西藏电力市场建设运营，维护西藏电力市场秩序和经营主体合法权益， 根据《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会令第 20 号）《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>REL-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-3D787AF073</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《重庆电力中长期市场实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>局华中监管局 Aa 字体： 小 | 中 | 大 为加快全国统一电力市场建设，进一步规范和完善重庆电力市场建设运营，维护重庆电力市场秩序和经营主体合法权益， 根据《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会令第20号）《国家发展改革委 国家能源局关于印发&lt;电力中长期市场基本规则&gt;的通知》（发改能源规〔2025〕1656号） 等文</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>REL-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-35BEAAF482</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《湖北省电力中长期市场实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>快推进全国统一电力市场体系建设，规范湖北电力中长期交易行为，依法维护湖北电力市场秩序、保护电力市场经营主体合法权益，保证电力市场的统一、开放、竞争、有序， 依据《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会令 2024 年第 20 号）、《国家发展改革委 国家能源局关于印发&lt;电力中长期市场基本规则&gt;的通知》（发改能源规 〔 20</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>REL-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-1A6D55E163</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《江西电力中长期市场实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>华中监管局 Aa 字体： 小 | 中 | 大 为加快全国统一电力市场建设，进一步规范和完善江西电力市场建设运营，维护江西电力市场秩序和经营主体合法权益， 根据 《电力市场运行基本规则》 （中华人民共和国国家发展和改革委员会令第 20 号）《国家发展改革委 国家能源局关于印发 &lt; 电力中长期市场基本规则 &gt; 的通知》（发改能源规〔 2025 〕</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>REL-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-08F5111897</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-7DF0C00260</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力并网运行管理实施细则》、《山东省电力辅助服务管理实施细则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2023-07-24</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>修订</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东省电力并网运行管理实施细则</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室 山东省电力并网运行与辅助服务管理实施细则修订稿 关于印发《山东省电力并网运行管理实</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>REL-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-F67BBBF923</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>【关于印发《电力中长期市场基本规则》的通知(发改能源规〔2025〕1656号)】-国家发展和改革委员会</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>中心有限公司、广州电力交易中心有限责任公司： 为贯彻落实加快建设全国统一电力市场要求，深化电力中长期市场建设，规范电力中长期交易行为，适应电力改革发展需要，根据《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会令2024年第20号）、《国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见》（发改体改〔2022〕118</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>REL-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-82D40D1344</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《西藏自治区电力中长期交易实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>明文引用</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>文号：国家发展改革委令第20号</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>REL-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-A3868601F8</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局华中监管局关于公开征求《重庆电力中长期交易实施细则（征求意见稿）》意见的通知</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>明文引用</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>文号：国家发展改革委令第20号</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>REL-0017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-DEDA1D301C</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>华中能源监管局关于公开征求《华中区域(东四省)省间电力互济市场交易规则》意见的通知</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>明文引用</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>文号：国家发展改革委令第20号</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>REL-0018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260425-2B6F6F94C5</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《山东电力市场规则(试行)》(征求意见稿)意见的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>管办公室 Aa 字体： 小 | 中 | 大 为贯彻落实《国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见》(发改体改〔2022〕118号)、《电力市场运行基本规则》(国家发改委2024年第20号令)、《国家发展改革委 国家能源局关于深化新能源上网电价市场化改革 促进新能源高质量发展的通知》(发改价格〔2025〕136号)等</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>REL-0019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-0D440B2FA1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《重庆市电力中长期交易规则》的通知</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>华中监能市场 ﹝ 2024 ﹞ 149 号 国网西南分部，国网重庆市电力公司，重庆电力交易中心有限公司，重庆市各有关发电企业、售电公司、电力用户 ： 为贯彻落实《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会第 20 号令）、 《国家发展改革委 国家能源局关于建立煤电容量电价机制的通知》（发改价格〔 2023 〕 1501 号）、</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>REL-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-2ABE953CDD</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局关于印发《电力市场注册基本规则》的通知</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2024-09-13</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260424-10A4BBBC6D</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：电力市场运行基本规则</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>《中共中央 国务院关于进一步深化电力体制改革的若干意见》《国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见》（发改体改〔2022〕118号）《电力市场运行基本规则》（中华人民共和国国家发展和改革委员会2024年第20号令）等文件，结合工作实际，制定本规则。 第二条 本规则所称电力市场包含电力中长期、现货、辅助服务市场等。</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>REL-0021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-CAE77C6F94</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东电力市场参数（试行）》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-CB9FE0315E</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东电力市场规则(试行)》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-19</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>文号：鲁监能市场规〔2024〕24号</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>国家能源局关于印发&lt;电力现货市场基本规则（试行）&gt;的通知》（发改能源规〔2023〕1217号）等文件要求，根据《关于印发&lt;山东电力市场规则（试行）&gt;的通知》（鲁监能市场规〔2024〕24号）规定，山东能源监管办会同省发展改革委、省能源局组织市场运营机构、电网企业和相关经营主体编制修订了《山东电力市场参数（试行）》，现予以印发。 一、《山东电力市场</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>REL-0022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-0A6267C300</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>关于征求《山东电力市场参数(试行)》(征求意见稿)意见的公告_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-19</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-CB9FE0315E</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东电力市场规则(试行)》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-19</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>修订</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>文号：鲁监能市场规〔2024〕24号</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>》(发改能源规〔2023〕1217号)等文件要求，山东能源监管办会同省发展改革委、省能源局组织市场运营机构和相关经营主体修订形成了《山东电力市场规则(试行)》(鲁监能市场规〔2024〕24号)。为适应电力市场运行需要，山东能源监管办会同省发展改革委、省能源局同步开展市场运行有关参数修订工作，经前期研究讨论，起草了《山东电力市场参数(试行)》(征求意</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>REL-0023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-0A6267C300</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>关于征求《山东电力市场参数(试行)》(征求意见稿)意见的公告_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-19</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-09ACA5D018</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>关于公开征求《山东电力市场规则(试行)》(征求意见稿)意见的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-08</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>修订</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东电力市场规则(试行</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>市场基本规则(试行)&gt;的通知》(发改能源规〔2023〕1217号)等文件要求，山东能源监管办会同省发展改革委、省能源局组织市场运营机构和相关经营主体修订形成了《山东电力市场规则(试行)》(鲁监能市场规〔2024〕24号)。为适应电力市场运行需要，山东能源监管办会同省发展改革委、省能源局同步开展市场运行有关参数修订工作，经前期研究讨论，起草了</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>REL-0024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-E982922381</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>关于修订《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2021-09-24</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-6EEB6D3357</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2021-04-30</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>修订</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东省电力中长期交易规则</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>关于修订《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室 关于修订《山东省电力中长期交易规则》的通知 2021-09-24 关于修订《山东省电力中长期交易规则》的通知_国家能源局山东监</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>REL-0025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-2E651E50F1</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>关于公示新增电力中长期交易发电企业(机组)名单的通知 - 2021年3号_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2021-09-22</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-6EEB6D3357</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2021-04-30</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东省电力中长期交易规则</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>长期交易发电企业(机组)名单的通知 - 2021年3号 2021-09-22 15:24 来源：国家能源局山东监管办公室 Aa 字体： 小 | 中 | 大 根据《山东省电力中长期交易规则》有关要求，我办对新申请参与电力中长期交易的发电企业(机组)进行了审核。现将符合市场准入基本条件的发电企业机组予以公示，公示时间为2021年9月17日至2020年</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>REL-0026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-B234995E67</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>关于公示新增电力中长期交易发电企业(机组)名单的通知 - 2021年2号_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2021-06-03</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-6EEB6D3357</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2021-04-30</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东省电力中长期交易规则</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>长期交易发电企业(机组)名单的通知 - 2021年2号 2021-06-03 14:42 来源：国家能源局山东监管办公室 Aa 字体： 小 | 中 | 大 根据《山东省电力中长期交易规则》、《山东省电力直接交易试点发电企业(机组)准入管理办法》和有关精神，我办对新申请参与电力中长期交易的发电企业(机组)进行了审核。现将符合市场准入基本条件的发电企</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>REL-0027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-46DA048C90</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>关于公示新增电力中长期交易发电企业(机组)名单的通知 - 2021年1号_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2021-05-20</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-20260426-6EEB6D3357</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>关于印发《山东省电力中长期交易规则》的通知_国家能源局山东监管办公室</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2021-04-30</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>引用依据</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>规则名称：山东省电力中长期交易规则</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>长期交易发电企业(机组)名单的通知 - 2021年1号 2021-05-20 17:00 来源：国家能源局山东监管办公室 Aa 字体： 小 | 中 | 大 根据《山东省电力中长期交易规则》、《山东省电力直接交易试点发电企业(机组)准入管理办法》和有关精神，我办对新申请参与电力中长期交易的发电企业(机组)进行了审核。现将符合市场准入基本条件的发电企</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>仅由新政策明文引用旧政策时生成</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -24934,7 +27729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27561,7 +30356,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32548,563 +35343,4 @@
   <autoFilter ref="A1:L80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>评测编号</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>问题</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>标准依据文件</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Top1资料编号</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Top1标题</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Top1得分</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Top3标题</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Top3命中</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>标准文件是否已入库</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Q-001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>全国统一电力市场体系建设的主要目标是什么</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>关于加快建设全国统一电力市场体系的指导意见</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-FD9AA2BEA1</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>49.00</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家能源局关于印发《电力市场注册基本规则》的通知</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Q-002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>电力市场注册基本规则对经营主体注册提出了哪些要求</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>电力市场注册基本规则</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-2ABE953CDD</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局关于印发《电力市场注册基本规则》的通知</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>47.00</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局关于印发《电力市场注册基本规则》的通知 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Q-003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>电力市场运行基本规则中市场成员包括哪些类型</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>电力市场运行基本规则</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-10A4BBBC6D</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>37.00</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>电力市场运行基本规则_国家发展和改革委员会_中国政府网 | 【关于建立全国统一电力市场评价制度的通知(发改办体改〔2025〕1032号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Q-004</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>省间电力现货交易规则修订主要涉及哪些内容</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>关于修订省间电力现货交易规则的复函</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-55178B2DFC</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>【关于修订省间电力现货交易规则的复函(发改办体改〔2026〕275号)】-国家发展和改革委员会</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>65.00</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>【关于修订省间电力现货交易规则的复函(发改办体改〔2026〕275号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Q-005</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>华中区域省间电力中长期市场实施细则适用于哪些交易范围</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>华中区域省间电力中长期市场实施细则</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-97CB3F74FC</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>国家能源局华中监管局关于印发《华中区域省间电力中长期市场实施细则》的通知 | 关于公开征求《华中区域省间电力中长期交易实施细则（征求意见稿）》意见的通知 | 关于印发《重庆市电力中长期市场实施细则》的通知</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Q-006</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>湖北省电力中长期市场实施细则规定了哪些主要交易类型</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>湖北省电力中长期市场实施细则</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-663B4D5B07</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>关于印发《湖北省电力中长期市场实施细则》的通知</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>49.00</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>关于印发《湖北省电力中长期市场实施细则》的通知</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Q-007</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>山东电力市场规则试行文件中中长期和现货如何衔接</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>山东电力市场规则(试行)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260426-2321F82FD1</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>关于山东电力现货市场由试运行转正式运行的通知_国家能源局山东监管办公室</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>31.50</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>关于山东电力现货市场由试运行转正式运行的通知_国家能源局山东监管办公室 | 《山东电力市场规则(试行)》编制说明_国家能源局山东监管办公室 | 关于印发《山东电力市场规则(试行)》的通知_国家能源局山东监管办公室</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Q-008</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>山东并网运行和辅助服务管理实施细则涉及哪些主体和费用机制</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>山东省电力并网运行管理实施细则;山东省电力辅助服务管理实施细则</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-08F5111897</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>43.00</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>关于印发《山东省电力并网运行管理实施细则》《山东省电力辅助服务管理实施细则》(修订稿)的通知_国家能源局山东监管办公室 | 关于印发《山东省电力并网运行管理实施细则》、《山东省电力辅助服务管理实施细则》的通知_国家能源局山东监管办公室 | 关于公开征求《山东省电力并网运行管理实施细则(征求意见稿)》《山东省电力辅助服务管理实施细则(征求意见稿)》意见的通知_国家能源局山东监管办公室</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Q-009</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>南方区域中长期电能量交易实施细则规定的交易组织方式有哪些</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>南方区域电力市场中长期电能量交易实施细则</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260424-E89DAD0775</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>南方区域电力市场中长期电能量交易实施细则等5项实施细则</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>40.50</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>南方区域电力市场中长期电能量交易实施细则等5项实施细则 | 关于加强辖区中长期批发交易合同签约履约监管的通知 | 电力市场信息披露基本规则（国能发监管〔2024〕9号）</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Q-010</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>辅助服务市场基本规则对辅助服务品种和结算提出了哪些要求</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>电力辅助服务市场基本规则</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>AUTO-20260425-54244C417B</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>【关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)】-国家发展和改革委员会</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>37.00</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>【关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)】-国家发展和改革委员会 | 国家发展改革委 国家能源局关于加快建设全国统一电力市场体系的指导意见_国务院部门文件_中国政府网 | 关于印发《电力辅助服务市场基本规则》的通知</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>